<commit_message>
Mejoras en el diseño responsivo
</commit_message>
<xml_diff>
--- a/excel/21-septiembre.xlsx
+++ b/excel/21-septiembre.xlsx
@@ -1,102 +1,65 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/87359f702c00cddf/Escritorio/Aniversario_Uniremington/semana-aniversario/excel/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="11_2B590B579470F02A6164AD51570AB8777BEFF481" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5B976192-2B72-4A8B-8833-1749D6418BD3}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="21-septiembre" sheetId="1" r:id="rId1"/>
+    <sheet name="21-septiembre" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'21-septiembre'!$A$1:$H$2</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'21-septiembre'!$1:$1</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
-  <extLst>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
-  </extLst>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
-  <si>
-    <t>Evento</t>
-  </si>
-  <si>
-    <t>Fecha</t>
-  </si>
-  <si>
-    <t>Hora</t>
-  </si>
-  <si>
-    <t>Lugar</t>
-  </si>
-  <si>
-    <t>Descripción</t>
-  </si>
-  <si>
-    <t>Participación</t>
-  </si>
-  <si>
-    <t>Fotografía</t>
-  </si>
-  <si>
-    <t>Observaciones</t>
-  </si>
-  <si>
-    <t>Apertura Uniremington Fest</t>
-  </si>
-  <si>
-    <t>21 de septiembre</t>
-  </si>
-  <si>
-    <t>Salon audivisual</t>
-  </si>
-  <si>
-    <t>Inicio de la semana de aniversario.</t>
-  </si>
-  <si>
-    <t>apertura.jpg</t>
-  </si>
-  <si>
-    <t>Asistencia de la comunidad universitaria.</t>
-  </si>
-  <si>
-    <t>si</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="6">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
+    </font>
+    <font>
+      <name val="Aptos Display"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Aptos"/>
+      <b val="1"/>
+      <color rgb="0017324D"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Aptos"/>
+      <color rgb="0017324D"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Aptos"/>
+      <b val="1"/>
+      <color rgb="00C84F42"/>
+      <sz val="10"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="6">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -106,8 +69,23 @@
         <fgColor rgb="FF0E4C92"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00164E63"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF1D6"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -124,36 +102,148 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <bottom style="thin">
+        <color rgb="00D7E4E8"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+  <cellXfs count="10">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="20" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="20" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="20" fontId="4" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2000250" cy="1333500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -440,74 +530,111 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00E76F51"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:H2"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="28"/>
   <cols>
-    <col min="1" max="1" width="45" customWidth="1"/>
-    <col min="2" max="2" width="20" customWidth="1"/>
-    <col min="3" max="3" width="18" customWidth="1"/>
-    <col min="4" max="4" width="22" customWidth="1"/>
-    <col min="5" max="5" width="55" customWidth="1"/>
-    <col min="6" max="6" width="22" customWidth="1"/>
-    <col min="7" max="7" width="24" customWidth="1"/>
-    <col min="8" max="8" width="30" customWidth="1"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="25" customWidth="1" min="4" max="4"/>
+    <col width="43" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="32" customWidth="1" min="7" max="7"/>
+    <col width="54" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Evento</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Fecha</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Hora</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Lugar</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Descripción</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Participación</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>Observaciones</t>
+        </is>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C2" s="3">
-        <v>0.60416666666666663</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="H2" t="s">
-        <v>13</v>
+    <row r="2" ht="112" customHeight="1">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>Apertura Uniremington Fest</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>21 de septiembre</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="n">
+        <v>0.6041666666666666</v>
+      </c>
+      <c r="D2" s="8" t="inlineStr">
+        <is>
+          <t>Salon audivisual</t>
+        </is>
+      </c>
+      <c r="E2" s="8" t="inlineStr">
+        <is>
+          <t>Inicio de la semana de aniversario.</t>
+        </is>
+      </c>
+      <c r="F2" s="9" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="G2" s="8" t="inlineStr">
+        <is>
+          <t>apertura.jpg</t>
+        </is>
+      </c>
+      <c r="H2" s="8" t="inlineStr">
+        <is>
+          <t>Asistencia de la comunidad universitaria.</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H2" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:H2"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>